<commit_message>
Robot sync: logs en cada paso + informe por correo al finalizar
- LogMessage en INICIO, SAP conectado, nº complementos/pendientes, cada CREATE y cada PLACA/REMOVE/ADD, FIN
- Al final arma resumen HTML (totales + errores) y lo envia por SMTP a MAIL_TO
- Config.xlsx: nuevas claves SMTP_SERVER/PORT/USER/PASS/MAIL_TO; si no hay SMTP_SERVER se omite (ContinueOnError)
- Requiere paquete UiPath.Mail.Activities

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/robot/SyncEdicionesCuadro.Config.sample.xlsx
+++ b/robot/SyncEdicionesCuadro.Config.sample.xlsx
@@ -66,7 +66,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -88,11 +88,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -102,6 +146,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -498,8 +544,8 @@
           <t>ENTORNO  —  PRD o QA. QA = SAP SBOFERCO_SANDBOX (probar aqui primero)</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="8" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -520,8 +566,8 @@
           <t>1) Credenciales SQL del OUTBOX  —  SERVER-APPS-TAB / Picking_Management (+ acceso al linked server [server-sql])</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -555,8 +601,8 @@
           <t>2) Login de la BD de SAP  —  DbUserName/DbPassword con que SAP abre la Company DB (NO el usuario B1)</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -590,8 +636,8 @@
           <t>3) Usuario de aplicacion SAP B1  —  El que consume licencia de Business One</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -625,8 +671,8 @@
           <t>Endpoints (no cambiar salvo migracion de server)</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -747,11 +793,94 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Informe por correo (SMTP)  —  servidor de correo saliente</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>SMTP_SERVER</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr"/>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Servidor SMTP (ej. el mismo de tus otros robots)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>SMTP_PORT</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>587</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Puerto SMTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>SMTP_USER</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr"/>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Usuario/remitente del correo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>SMTP_PASS</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Contrasena del remitente</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>MAIL_TO</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>pedro.morales@ferco.com.gt</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Destinatario(s) del informe (separar con ;)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Robot sync: quitar informe por correo, dejar solo logs
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/robot/SyncEdicionesCuadro.Config.sample.xlsx
+++ b/robot/SyncEdicionesCuadro.Config.sample.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -793,94 +793,12 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Informe por correo (SMTP)  —  servidor de correo saliente</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>SMTP_SERVER</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr"/>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Servidor SMTP (ej. el mismo de tus otros robots)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>SMTP_PORT</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>587</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Puerto SMTP</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>SMTP_USER</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr"/>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Usuario/remitente del correo</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>SMTP_PASS</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr"/>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Contrasena del remitente</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>MAIL_TO</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>pedro.morales@ferco.com.gt</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Destinatario(s) del informe (separar con ;)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>

</xml_diff>